<commit_message>
add new combined vocab rdf exports, use in general vocab export command, update exports
</commit_message>
<xml_diff>
--- a/storage/app/public/vocabs/analogue/1.3/analogue_1-3.xlsx
+++ b/storage/app/public/vocabs/analogue/1.3/analogue_1-3.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1351">
   <si>
     <t>synonyms</t>
   </si>
@@ -2915,7 +2915,7 @@
     <t>laser vibrometer</t>
   </si>
   <si>
-    <t>#laser vibrometre</t>
+    <t>#laser vibrometre#vibrometer#vibrometre#polytec vibrometer</t>
   </si>
   <si>
     <t>https://epos-msl.uu.nl/voc/analoguemodelling/1.3/ancillary_equipment-model_structure_monitoring_3d-acoustic_measurement_-_active_source-laser_vibrometer</t>
@@ -3651,6 +3651,33 @@
   </si>
   <si>
     <t>https://epos-msl.uu.nl/voc/analoguemodelling/1.3/software-digital_image_correlation_dic-particle_image_velocimetry_piv</t>
+  </si>
+  <si>
+    <t>PIV - MatPIV</t>
+  </si>
+  <si>
+    <t>#matpiv</t>
+  </si>
+  <si>
+    <t>https://epos-msl.uu.nl/voc/analoguemodelling/1.3/software-digital_image_correlation_dic-particle_image_velocimetry_piv-piv_-_matpiv</t>
+  </si>
+  <si>
+    <t>PIV - PIVlab</t>
+  </si>
+  <si>
+    <t>#pivlab#pivlab software</t>
+  </si>
+  <si>
+    <t>https://epos-msl.uu.nl/voc/analoguemodelling/1.3/software-digital_image_correlation_dic-particle_image_velocimetry_piv-piv_-_pivlab</t>
+  </si>
+  <si>
+    <t>PIV - TecPIV</t>
+  </si>
+  <si>
+    <t>#tecpiv</t>
+  </si>
+  <si>
+    <t>https://epos-msl.uu.nl/voc/analoguemodelling/1.3/software-digital_image_correlation_dic-particle_image_velocimetry_piv-piv_-_tecpiv</t>
   </si>
   <si>
     <t>structure from motion (SfM)</t>
@@ -4380,7 +4407,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I664"/>
+  <dimension ref="A1:I667"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -9438,7 +9465,7 @@
       </c>
     </row>
     <row r="605" spans="1:9">
-      <c r="B605" t="s">
+      <c r="D605" t="s">
         <v>1212</v>
       </c>
       <c r="F605" t="s">
@@ -9449,7 +9476,7 @@
       </c>
     </row>
     <row r="606" spans="1:9">
-      <c r="C606" t="s">
+      <c r="D606" t="s">
         <v>1215</v>
       </c>
       <c r="F606" t="s">
@@ -9460,7 +9487,7 @@
       </c>
     </row>
     <row r="607" spans="1:9">
-      <c r="C607" t="s">
+      <c r="D607" t="s">
         <v>1218</v>
       </c>
       <c r="F607" t="s">
@@ -9471,7 +9498,7 @@
       </c>
     </row>
     <row r="608" spans="1:9">
-      <c r="C608" t="s">
+      <c r="B608" t="s">
         <v>1221</v>
       </c>
       <c r="F608" t="s">
@@ -9537,414 +9564,447 @@
       </c>
     </row>
     <row r="614" spans="1:9">
-      <c r="B614" t="s">
+      <c r="C614" t="s">
         <v>1239</v>
       </c>
+      <c r="F614" t="s">
+        <v>1240</v>
+      </c>
       <c r="G614" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="615" spans="1:9">
-      <c r="B615" t="s">
-        <v>1241</v>
+      <c r="C615" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F615" t="s">
+        <v>1243</v>
       </c>
       <c r="G615" t="s">
-        <v>1242</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="616" spans="1:9">
-      <c r="B616" t="s">
-        <v>1243</v>
+      <c r="C616" t="s">
+        <v>1245</v>
+      </c>
+      <c r="F616" t="s">
+        <v>1246</v>
       </c>
       <c r="G616" t="s">
-        <v>1244</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="617" spans="1:9">
       <c r="B617" t="s">
-        <v>1245</v>
+        <v>1248</v>
       </c>
       <c r="G617" t="s">
-        <v>1246</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="618" spans="1:9">
       <c r="B618" t="s">
-        <v>1247</v>
+        <v>1250</v>
       </c>
       <c r="G618" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="619" spans="1:9">
       <c r="B619" t="s">
-        <v>1249</v>
+        <v>1252</v>
       </c>
       <c r="G619" t="s">
-        <v>1250</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="620" spans="1:9">
       <c r="B620" t="s">
-        <v>1251</v>
+        <v>1254</v>
       </c>
       <c r="G620" t="s">
-        <v>1252</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="621" spans="1:9">
       <c r="B621" t="s">
-        <v>1253</v>
+        <v>1256</v>
       </c>
       <c r="G621" t="s">
-        <v>1254</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="622" spans="1:9">
       <c r="B622" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
       <c r="G622" t="s">
-        <v>1256</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="623" spans="1:9">
       <c r="B623" t="s">
-        <v>1257</v>
+        <v>1260</v>
       </c>
       <c r="G623" t="s">
-        <v>1258</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="624" spans="1:9">
       <c r="B624" t="s">
-        <v>1259</v>
+        <v>1262</v>
       </c>
       <c r="G624" t="s">
-        <v>1260</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="625" spans="1:9">
       <c r="B625" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="G625" t="s">
-        <v>1262</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="626" spans="1:9">
       <c r="B626" t="s">
-        <v>1263</v>
+        <v>1266</v>
       </c>
       <c r="G626" t="s">
-        <v>1264</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="627" spans="1:9">
       <c r="B627" t="s">
-        <v>1265</v>
+        <v>1268</v>
       </c>
       <c r="G627" t="s">
-        <v>1266</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="628" spans="1:9">
       <c r="B628" t="s">
-        <v>1267</v>
+        <v>1270</v>
       </c>
       <c r="G628" t="s">
-        <v>1268</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="629" spans="1:9">
       <c r="B629" t="s">
-        <v>1269</v>
+        <v>1272</v>
       </c>
       <c r="G629" t="s">
-        <v>1270</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="630" spans="1:9">
       <c r="B630" t="s">
-        <v>1271</v>
+        <v>1274</v>
       </c>
       <c r="G630" t="s">
-        <v>1272</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="631" spans="1:9">
       <c r="B631" t="s">
-        <v>1273</v>
+        <v>1276</v>
       </c>
       <c r="G631" t="s">
-        <v>1274</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="632" spans="1:9">
       <c r="B632" t="s">
-        <v>1275</v>
+        <v>1278</v>
       </c>
       <c r="G632" t="s">
-        <v>1276</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="633" spans="1:9">
       <c r="B633" t="s">
-        <v>1277</v>
+        <v>1280</v>
       </c>
       <c r="G633" t="s">
-        <v>1278</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="634" spans="1:9">
       <c r="B634" t="s">
-        <v>1279</v>
+        <v>1282</v>
       </c>
       <c r="G634" t="s">
-        <v>1280</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="635" spans="1:9">
       <c r="B635" t="s">
-        <v>1281</v>
+        <v>1284</v>
       </c>
       <c r="G635" t="s">
-        <v>1282</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="636" spans="1:9">
       <c r="B636" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="G636" t="s">
-        <v>1284</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="637" spans="1:9">
       <c r="B637" t="s">
-        <v>1285</v>
+        <v>1288</v>
       </c>
       <c r="G637" t="s">
-        <v>1286</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="638" spans="1:9">
       <c r="B638" t="s">
-        <v>1287</v>
+        <v>1290</v>
       </c>
       <c r="G638" t="s">
-        <v>1288</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="639" spans="1:9">
       <c r="B639" t="s">
-        <v>1289</v>
+        <v>1292</v>
       </c>
       <c r="G639" t="s">
-        <v>1290</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="640" spans="1:9">
       <c r="B640" t="s">
-        <v>1291</v>
+        <v>1294</v>
       </c>
       <c r="G640" t="s">
-        <v>1292</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="641" spans="1:9">
       <c r="B641" t="s">
-        <v>1293</v>
+        <v>1296</v>
       </c>
       <c r="G641" t="s">
-        <v>1294</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="642" spans="1:9">
       <c r="B642" t="s">
-        <v>1295</v>
-      </c>
-      <c r="F642" t="s">
-        <v>1296</v>
+        <v>1298</v>
       </c>
       <c r="G642" t="s">
-        <v>1297</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="643" spans="1:9">
       <c r="B643" t="s">
-        <v>1298</v>
+        <v>1300</v>
       </c>
       <c r="G643" t="s">
-        <v>1299</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="644" spans="1:9">
       <c r="B644" t="s">
-        <v>1300</v>
+        <v>1302</v>
       </c>
       <c r="G644" t="s">
-        <v>1301</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="645" spans="1:9">
       <c r="B645" t="s">
-        <v>1302</v>
+        <v>1304</v>
+      </c>
+      <c r="F645" t="s">
+        <v>1305</v>
       </c>
       <c r="G645" t="s">
-        <v>1303</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="646" spans="1:9">
       <c r="B646" t="s">
-        <v>1304</v>
+        <v>1307</v>
       </c>
       <c r="G646" t="s">
-        <v>1305</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="647" spans="1:9">
       <c r="B647" t="s">
-        <v>1306</v>
+        <v>1309</v>
       </c>
       <c r="G647" t="s">
-        <v>1307</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="648" spans="1:9">
       <c r="B648" t="s">
-        <v>1308</v>
+        <v>1311</v>
       </c>
       <c r="G648" t="s">
-        <v>1309</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="649" spans="1:9">
       <c r="B649" t="s">
-        <v>1310</v>
+        <v>1313</v>
       </c>
       <c r="G649" t="s">
-        <v>1311</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="650" spans="1:9">
       <c r="B650" t="s">
-        <v>1312</v>
+        <v>1315</v>
       </c>
       <c r="G650" t="s">
-        <v>1313</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="651" spans="1:9">
       <c r="B651" t="s">
-        <v>1314</v>
+        <v>1317</v>
       </c>
       <c r="G651" t="s">
-        <v>1315</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="652" spans="1:9">
       <c r="B652" t="s">
-        <v>1316</v>
+        <v>1319</v>
       </c>
       <c r="G652" t="s">
-        <v>1317</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="653" spans="1:9">
       <c r="B653" t="s">
-        <v>1318</v>
+        <v>1321</v>
       </c>
       <c r="G653" t="s">
-        <v>1319</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="654" spans="1:9">
       <c r="B654" t="s">
-        <v>1320</v>
+        <v>1323</v>
       </c>
       <c r="G654" t="s">
-        <v>1321</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="655" spans="1:9">
       <c r="B655" t="s">
-        <v>1322</v>
+        <v>1325</v>
       </c>
       <c r="G655" t="s">
-        <v>1323</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="656" spans="1:9">
       <c r="B656" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="G656" t="s">
-        <v>1325</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="657" spans="1:9">
       <c r="B657" t="s">
-        <v>1326</v>
+        <v>1329</v>
       </c>
       <c r="G657" t="s">
-        <v>1327</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="658" spans="1:9">
       <c r="B658" t="s">
-        <v>1328</v>
+        <v>1331</v>
       </c>
       <c r="G658" t="s">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="659" spans="1:9">
       <c r="B659" t="s">
-        <v>1330</v>
+        <v>1333</v>
       </c>
       <c r="G659" t="s">
-        <v>1331</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="660" spans="1:9">
       <c r="B660" t="s">
-        <v>1332</v>
+        <v>1335</v>
       </c>
       <c r="G660" t="s">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="661" spans="1:9">
       <c r="B661" t="s">
-        <v>1334</v>
+        <v>1337</v>
       </c>
       <c r="G661" t="s">
-        <v>1335</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="662" spans="1:9">
       <c r="B662" t="s">
-        <v>1336</v>
+        <v>1339</v>
       </c>
       <c r="G662" t="s">
-        <v>1337</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="663" spans="1:9">
       <c r="B663" t="s">
-        <v>1338</v>
+        <v>1341</v>
       </c>
       <c r="G663" t="s">
-        <v>1339</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="664" spans="1:9">
       <c r="B664" t="s">
-        <v>1340</v>
+        <v>1343</v>
       </c>
       <c r="G664" t="s">
-        <v>1341</v>
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="665" spans="1:9">
+      <c r="B665" t="s">
+        <v>1345</v>
+      </c>
+      <c r="G665" t="s">
+        <v>1346</v>
+      </c>
+    </row>
+    <row r="666" spans="1:9">
+      <c r="B666" t="s">
+        <v>1347</v>
+      </c>
+      <c r="G666" t="s">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="667" spans="1:9">
+      <c r="B667" t="s">
+        <v>1349</v>
+      </c>
+      <c r="G667" t="s">
+        <v>1350</v>
       </c>
     </row>
   </sheetData>

</xml_diff>